<commit_message>
Add synthetic cell-count example and QMP outputs
</commit_message>
<xml_diff>
--- a/example/reference_results/9_phyloseq_object/GTDB/phyloseq_summary_gtdb.xlsx
+++ b/example/reference_results/9_phyloseq_object/GTDB/phyloseq_summary_gtdb.xlsx
@@ -6,11 +6,15 @@
     <workbookView xWindow="0" yWindow="0" windowWidth="13125" windowHeight="6105" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Tax_Summary" sheetId="3" state="visible" r:id="rId1"/>
+    <sheet name="Tax_Summary" sheetId="7" state="visible" r:id="rId1"/>
     <sheet name="Top_Genera_Raw" sheetId="1" state="visible" r:id="rId2"/>
-    <sheet name="Sample_Stats_Raw" sheetId="2" state="visible" r:id="rId3"/>
-    <sheet name="Run_Provenance" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Column_Dictionary" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Top_Genera_CN_Corrected" sheetId="2" state="visible" r:id="rId3"/>
+    <sheet name="Top_Genera_ML_Corrected" sheetId="3" state="visible" r:id="rId4"/>
+    <sheet name="Sample_Stats_Raw" sheetId="4" state="visible" r:id="rId5"/>
+    <sheet name="Sample_Stats_CN_Corrected" sheetId="5" state="visible" r:id="rId6"/>
+    <sheet name="Sample_Stats_ML_Corrected" sheetId="6" state="visible" r:id="rId7"/>
+    <sheet name="Run_Provenance" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Column_Dictionary" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
 </workbook>
 </file>
@@ -157,7 +161,7 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">Sample name as stored in the phyloseq object (sample_names()).</t>
+          <t xml:space="preserve">Integer rank (1 = most abundant) of this genus among the top n_top_taxa CLASSIFIED genera by summed abundance within its taxonomy database x abundance source combination -- ASVs with an unclassified (NA) Genus assignment are excluded from this ranking (see the Identify Top Genera section). Row order in the sheet already reflects this rank.</t>
         </r>
       </text>
     </comment>
@@ -169,7 +173,7 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">Total abundance summed across ASVs for this sample, i.e. sample_sums(). Units follow the source table: reads, copy-number-corrected abundance, or microbial-load-scaled abundance. Raw counts are whole numbers of reads; copy-number-corrected and microbial-load-corrected values are rounded to 1 decimal place.</t>
+          <t xml:space="preserve">Identifier of the representative ASV that tax_glom() retained for this genus after collapsing all ASVs sharing the same Genus assignment into a single aggregated row.</t>
         </r>
       </text>
     </comment>
@@ -181,7 +185,7 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">Number of ASVs with a non-zero count in this sample — the observed taxa richness for that sample.</t>
+          <t xml:space="preserve">Genus-level taxonomic assignment for this aggregated group, taken from the Genus column of the taxonomy table. Never NA in this sheet, since unclassified genera are excluded from the top-N ranking.</t>
         </r>
       </text>
     </comment>
@@ -193,7 +197,19 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">Total_Abundance for this sample expressed as a percentage of summed Total_Abundance across all samples in the same taxonomy database x abundance source combination, rounded to 2 decimal places.</t>
+          <t xml:space="preserve">Total abundance summed across all samples for this genus, i.e. taxa_sums() on the genus-aggregated phyloseq object. Units follow the source table: reads, copy-number-corrected abundance, or microbial-load-scaled abundance. Raw counts are whole numbers of reads; copy-number-corrected and microbial-load-corrected values are rounded to 1 decimal place.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Total_Abundance for this genus expressed as a percentage of the summed abundance of ALL genera (including any unclassified/NA genus) in the same taxonomy database x abundance source combination, rounded to 2 decimal places -- i.e. a true share of the whole community, not just of the classified fraction.</t>
         </r>
       </text>
     </comment>
@@ -215,6 +231,250 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
+          <t xml:space="preserve">Integer rank (1 = most abundant) of this genus among the top n_top_taxa CLASSIFIED genera by summed abundance within its taxonomy database x abundance source combination -- ASVs with an unclassified (NA) Genus assignment are excluded from this ranking (see the Identify Top Genera section). Row order in the sheet already reflects this rank.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Identifier of the representative ASV that tax_glom() retained for this genus after collapsing all ASVs sharing the same Genus assignment into a single aggregated row.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Genus-level taxonomic assignment for this aggregated group, taken from the Genus column of the taxonomy table. Never NA in this sheet, since unclassified genera are excluded from the top-N ranking.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Total abundance summed across all samples for this genus, i.e. taxa_sums() on the genus-aggregated phyloseq object. Units follow the source table: reads, copy-number-corrected abundance, or microbial-load-scaled abundance. Raw counts are whole numbers of reads; copy-number-corrected and microbial-load-corrected values are rounded to 1 decimal place.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Total_Abundance for this genus expressed as a percentage of the summed abundance of ALL genera (including any unclassified/NA genus) in the same taxonomy database x abundance source combination, rounded to 2 decimal places -- i.e. a true share of the whole community, not just of the classified fraction.</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments5.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author/>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Sample name as stored in the phyloseq object (sample_names()).</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Total abundance summed across ASVs for this sample, i.e. sample_sums(). Units follow the source table: reads, copy-number-corrected abundance, or microbial-load-scaled abundance. Raw counts are whole numbers of reads; copy-number-corrected and microbial-load-corrected values are rounded to 1 decimal place.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Number of ASVs with a non-zero count in this sample — the observed taxa richness for that sample.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Total_Abundance for this sample expressed as a percentage of summed Total_Abundance across all samples in the same taxonomy database x abundance source combination, rounded to 2 decimal places.</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments6.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author/>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Sample name as stored in the phyloseq object (sample_names()).</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Total abundance summed across ASVs for this sample, i.e. sample_sums(). Units follow the source table: reads, copy-number-corrected abundance, or microbial-load-scaled abundance. Raw counts are whole numbers of reads; copy-number-corrected and microbial-load-corrected values are rounded to 1 decimal place.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Number of ASVs with a non-zero count in this sample — the observed taxa richness for that sample.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Total_Abundance for this sample expressed as a percentage of summed Total_Abundance across all samples in the same taxonomy database x abundance source combination, rounded to 2 decimal places.</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments7.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author/>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Sample name as stored in the phyloseq object (sample_names()).</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Total abundance summed across ASVs for this sample, i.e. sample_sums(). Units follow the source table: reads, copy-number-corrected abundance, or microbial-load-scaled abundance. Raw counts are whole numbers of reads; copy-number-corrected and microbial-load-corrected values are rounded to 1 decimal place.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Number of ASVs with a non-zero count in this sample — the observed taxa richness for that sample.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Total_Abundance for this sample expressed as a percentage of summed Total_Abundance across all samples in the same taxonomy database x abundance source combination, rounded to 2 decimal places.</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments8.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author/>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
           <t xml:space="preserve">Generation timestamp with timezone.</t>
         </r>
       </text>
@@ -428,7 +688,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="142">
   <si>
     <t xml:space="preserve">Rank</t>
   </si>
@@ -457,6 +717,12 @@
     <t xml:space="preserve">Bacteroides</t>
   </si>
   <si>
+    <t xml:space="preserve">ASV8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alistipes</t>
+  </si>
+  <si>
     <t xml:space="preserve">ASV11</t>
   </si>
   <si>
@@ -499,10 +765,19 @@
     <t xml:space="preserve">Limosilactobacillus</t>
   </si>
   <si>
-    <t xml:space="preserve">ASV25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UBA7185</t>
+    <t xml:space="preserve">ASV22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brotaphodocola</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ASV28</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ASV53</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Helicobacter</t>
   </si>
   <si>
     <t xml:space="preserve">SampleID</t>
@@ -655,7 +930,7 @@
     <t xml:space="preserve">R_Version</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-09-29 14:59:59 CEST</t>
+    <t xml:space="preserve">2026-09-29 15:16:34 CEST</t>
   </si>
   <si>
     <t xml:space="preserve">GTDB_raw_counts</t>
@@ -670,7 +945,7 @@
     <t xml:space="preserve">/Users/amro/Documents/workflows/DADA2_16S_Illumina_PairedEnd_Workflow/example/run_results/5_dada2_pipeline/gtdb_taxonomy_table.csv</t>
   </si>
   <si>
-    <t xml:space="preserve">e823c3994794149e0523f1df8986cb1e</t>
+    <t xml:space="preserve">d751e4a9c7f712adbe7998b3a352a42f</t>
   </si>
   <si>
     <t xml:space="preserve">/Users/amro/Documents/workflows/DADA2_16S_Illumina_PairedEnd_Workflow/example/data/metadata.tsv</t>
@@ -685,6 +960,36 @@
     <t xml:space="preserve">R version 4.5.2 (2025-10-31)</t>
   </si>
   <si>
+    <t xml:space="preserve">GTDB_copy_number_corrected</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/Users/amro/Documents/workflows/DADA2_16S_Illumina_PairedEnd_Workflow/example/run_results/7_copy_number_correction/copy_number_corrected_asv_count_table.csv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">c947e7664fb75efd061c5c8de721b7e8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/Users/amro/Documents/workflows/DADA2_16S_Illumina_PairedEnd_Workflow/example/run_results/7_copy_number_correction/copy_number_correction_summary.xlsx</t>
+  </si>
+  <si>
+    <t xml:space="preserve">143355f48ec0fd4be6486a49b09480fa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GTDB_microbial_load_corrected</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/Users/amro/Documents/workflows/DADA2_16S_Illumina_PairedEnd_Workflow/example/run_results/8_microbial_load_correction/microbial_load_corrected_abundance_table.csv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">055887ea8e51ec34a9a0f51d6d4df72f</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/Users/amro/Documents/workflows/DADA2_16S_Illumina_PairedEnd_Workflow/example/run_results/8_microbial_load_correction/microbial_load_correction_summary.xlsx</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bd25f596934f17d031f57b031d8971ab</t>
+  </si>
+  <si>
     <t xml:space="preserve">Sheet</t>
   </si>
   <si>
@@ -769,6 +1074,12 @@
     <t xml:space="preserve">Total_Abundance for this genus expressed as a percentage of the summed abundance of ALL genera (including any unclassified/NA genus) in the same taxonomy database x abundance source combination, rounded to 2 decimal places -- i.e. a true share of the whole community, not just of the classified fraction.</t>
   </si>
   <si>
+    <t xml:space="preserve">Top_Genera_CN_Corrected</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Top_Genera_ML_Corrected</t>
+  </si>
+  <si>
     <t xml:space="preserve">Sample_Stats_Raw</t>
   </si>
   <si>
@@ -782,6 +1093,12 @@
   </si>
   <si>
     <t xml:space="preserve">Total_Abundance for this sample expressed as a percentage of summed Total_Abundance across all samples in the same taxonomy database x abundance source combination, rounded to 2 decimal places.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sample_Stats_CN_Corrected</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sample_Stats_ML_Corrected</t>
   </si>
   <si>
     <t xml:space="preserve">Tax_Summary</t>
@@ -852,8 +1169,47 @@
 </styleSheet>
 </file>
 
+<file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="Table10" displayName="Table10" ref="A1:R4" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:R4"/>
+  <tableColumns count="18">
+    <tableColumn id="1" name="Generated_At"/>
+    <tableColumn id="2" name="Combination"/>
+    <tableColumn id="3" name="Abundance_File"/>
+    <tableColumn id="4" name="Abundance_MD5"/>
+    <tableColumn id="5" name="Provenance_File"/>
+    <tableColumn id="6" name="Provenance_MD5"/>
+    <tableColumn id="7" name="Taxonomy_File"/>
+    <tableColumn id="8" name="Taxonomy_MD5"/>
+    <tableColumn id="9" name="Metadata_File"/>
+    <tableColumn id="10" name="Metadata_MD5"/>
+    <tableColumn id="11" name="Tree_File"/>
+    <tableColumn id="12" name="Tree_MD5"/>
+    <tableColumn id="13" name="Input_ASVs"/>
+    <tableColumn id="14" name="Taxonomy_Matched_ASVs"/>
+    <tableColumn id="15" name="Final_ASVs"/>
+    <tableColumn id="16" name="Top_Taxa"/>
+    <tableColumn id="17" name="Phyloseq_Version"/>
+    <tableColumn id="18" name="R_Version"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="Table11" displayName="Table11" ref="A1:C50" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:C50"/>
+  <tableColumns count="3">
+    <tableColumn id="1" name="Sheet"/>
+    <tableColumn id="2" name="Column"/>
+    <tableColumn id="3" name="Explanation"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table5" displayName="Table5" ref="A1:D8" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table9" displayName="Table9" ref="A1:D8" totalsRowCount="0" totalsRowShown="0">
   <autoFilter ref="A1:D8"/>
   <tableColumns count="4">
     <tableColumn id="1" name="Rank"/>
@@ -880,7 +1236,35 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="Table4" displayName="Table4" ref="A1:D21" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="Table4" displayName="Table4" ref="A1:E11" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:E11"/>
+  <tableColumns count="5">
+    <tableColumn id="1" name="Rank"/>
+    <tableColumn id="2" name="ASV_ID"/>
+    <tableColumn id="3" name="Genus"/>
+    <tableColumn id="4" name="Total_Abundance"/>
+    <tableColumn id="5" name="Relative_Abundance"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="Table5" displayName="Table5" ref="A1:E11" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:E11"/>
+  <tableColumns count="5">
+    <tableColumn id="1" name="Rank"/>
+    <tableColumn id="2" name="ASV_ID"/>
+    <tableColumn id="3" name="Genus"/>
+    <tableColumn id="4" name="Total_Abundance"/>
+    <tableColumn id="5" name="Relative_Abundance"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="Table6" displayName="Table6" ref="A1:D21" totalsRowCount="0" totalsRowShown="0">
   <autoFilter ref="A1:D21"/>
   <tableColumns count="4">
     <tableColumn id="1" name="SampleID"/>
@@ -892,40 +1276,27 @@
 </table>
 </file>
 
-<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="Table6" displayName="Table6" ref="A1:R2" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:R2"/>
-  <tableColumns count="18">
-    <tableColumn id="1" name="Generated_At"/>
-    <tableColumn id="2" name="Combination"/>
-    <tableColumn id="3" name="Abundance_File"/>
-    <tableColumn id="4" name="Abundance_MD5"/>
-    <tableColumn id="5" name="Provenance_File"/>
-    <tableColumn id="6" name="Provenance_MD5"/>
-    <tableColumn id="7" name="Taxonomy_File"/>
-    <tableColumn id="8" name="Taxonomy_MD5"/>
-    <tableColumn id="9" name="Metadata_File"/>
-    <tableColumn id="10" name="Metadata_MD5"/>
-    <tableColumn id="11" name="Tree_File"/>
-    <tableColumn id="12" name="Tree_MD5"/>
-    <tableColumn id="13" name="Input_ASVs"/>
-    <tableColumn id="14" name="Taxonomy_Matched_ASVs"/>
-    <tableColumn id="15" name="Final_ASVs"/>
-    <tableColumn id="16" name="Top_Taxa"/>
-    <tableColumn id="17" name="Phyloseq_Version"/>
-    <tableColumn id="18" name="R_Version"/>
+<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="Table7" displayName="Table7" ref="A1:D21" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:D21"/>
+  <tableColumns count="4">
+    <tableColumn id="1" name="SampleID"/>
+    <tableColumn id="2" name="Total_Abundance"/>
+    <tableColumn id="3" name="Observed_ASVs"/>
+    <tableColumn id="4" name="Pct_Total_Abundance"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
-<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="Table7" displayName="Table7" ref="A1:C32" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:C32"/>
-  <tableColumns count="3">
-    <tableColumn id="1" name="Sheet"/>
-    <tableColumn id="2" name="Column"/>
-    <tableColumn id="3" name="Explanation"/>
+<file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="Table8" displayName="Table8" ref="A1:D21" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:D21"/>
+  <tableColumns count="4">
+    <tableColumn id="1" name="SampleID"/>
+    <tableColumn id="2" name="Total_Abundance"/>
+    <tableColumn id="3" name="Observed_ASVs"/>
+    <tableColumn id="4" name="Pct_Total_Abundance"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1211,7 +1582,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <sheetPr>
-    <tabColor rgb="FFAF7AA1"/>
+    <tabColor rgb="FFEDC949"/>
   </sheetPr>
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
@@ -1227,18 +1598,18 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="B2" t="n">
         <v>1</v>
@@ -1252,35 +1623,35 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="B3" t="n">
         <v>11</v>
       </c>
       <c r="C3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D3" t="n">
-        <v>98.3</v>
+        <v>98.7</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="B4" t="n">
         <v>14</v>
       </c>
       <c r="C4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D4" t="n">
-        <v>98.3</v>
+        <v>98.7</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="B5" t="n">
         <v>26</v>
@@ -1294,16 +1665,16 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="B6" t="n">
         <v>43</v>
       </c>
       <c r="C6" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D6" t="n">
-        <v>94.8</v>
+        <v>95.3</v>
       </c>
     </row>
     <row r="7">
@@ -1311,21 +1682,21 @@
         <v>2</v>
       </c>
       <c r="B7" t="n">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C7" t="n">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D7" t="n">
-        <v>46.6</v>
+        <v>47</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="B8" t="n">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C8" t="n">
         <v>0</v>
@@ -1421,10 +1792,10 @@
         <v>10</v>
       </c>
       <c r="D4" t="n">
-        <v>3065</v>
+        <v>5318</v>
       </c>
       <c r="E4" t="n">
-        <v>2.47</v>
+        <v>4.28</v>
       </c>
     </row>
     <row r="5">
@@ -1438,10 +1809,10 @@
         <v>12</v>
       </c>
       <c r="D5" t="n">
-        <v>2036</v>
+        <v>3065</v>
       </c>
       <c r="E5" t="n">
-        <v>1.64</v>
+        <v>2.47</v>
       </c>
     </row>
     <row r="6">
@@ -1455,10 +1826,10 @@
         <v>14</v>
       </c>
       <c r="D6" t="n">
-        <v>1503</v>
+        <v>2036</v>
       </c>
       <c r="E6" t="n">
-        <v>1.21</v>
+        <v>1.64</v>
       </c>
     </row>
     <row r="7">
@@ -1472,10 +1843,10 @@
         <v>16</v>
       </c>
       <c r="D7" t="n">
-        <v>1415</v>
+        <v>1503</v>
       </c>
       <c r="E7" t="n">
-        <v>1.14</v>
+        <v>1.21</v>
       </c>
     </row>
     <row r="8">
@@ -1489,10 +1860,10 @@
         <v>18</v>
       </c>
       <c r="D8" t="n">
-        <v>1244</v>
+        <v>1415</v>
       </c>
       <c r="E8" t="n">
-        <v>1</v>
+        <v>1.14</v>
       </c>
     </row>
     <row r="9">
@@ -1506,10 +1877,10 @@
         <v>20</v>
       </c>
       <c r="D9" t="n">
-        <v>1199</v>
+        <v>1244</v>
       </c>
       <c r="E9" t="n">
-        <v>0.97</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -1523,10 +1894,10 @@
         <v>22</v>
       </c>
       <c r="D10" t="n">
-        <v>1028</v>
+        <v>1199</v>
       </c>
       <c r="E10" t="n">
-        <v>0.83</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="11">
@@ -1540,10 +1911,10 @@
         <v>24</v>
       </c>
       <c r="D11" t="n">
-        <v>823</v>
+        <v>1028</v>
       </c>
       <c r="E11" t="n">
-        <v>0.66</v>
+        <v>0.83</v>
       </c>
     </row>
   </sheetData>
@@ -1557,6 +1928,430 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <sheetPr>
+    <tabColor rgb="FFEDC949"/>
+  </sheetPr>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <cols>
+    <col min="1" max="1" width="4.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="6.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="19.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="15.71" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="18.71" hidden="0" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" t="n">
+        <v>8064</v>
+      </c>
+      <c r="E2" t="n">
+        <v>7.16</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" t="n">
+        <v>3065</v>
+      </c>
+      <c r="E3" t="n">
+        <v>2.72</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4" t="n">
+        <v>2659</v>
+      </c>
+      <c r="E4" t="n">
+        <v>2.36</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" t="n">
+        <v>2036</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1.81</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" t="s">
+        <v>16</v>
+      </c>
+      <c r="D6" t="n">
+        <v>1503</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1.34</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7" t="n">
+        <v>1244</v>
+      </c>
+      <c r="E7" t="n">
+        <v>1.11</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>21</v>
+      </c>
+      <c r="C8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8" t="n">
+        <v>1199</v>
+      </c>
+      <c r="E8" t="n">
+        <v>1.07</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>7</v>
+      </c>
+      <c r="C9" t="s">
+        <v>8</v>
+      </c>
+      <c r="D9" t="n">
+        <v>1176</v>
+      </c>
+      <c r="E9" t="n">
+        <v>1.04</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>23</v>
+      </c>
+      <c r="C10" t="s">
+        <v>24</v>
+      </c>
+      <c r="D10" t="n">
+        <v>1028</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.91</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>25</v>
+      </c>
+      <c r="C11" t="s">
+        <v>26</v>
+      </c>
+      <c r="D11" t="n">
+        <v>947</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.84</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+  <legacyDrawing r:id="rIdvml"/>
+  <tableParts count="1">
+    <tablePart r:id="rId5"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <sheetPr>
+    <tabColor rgb="FFAF7AA1"/>
+  </sheetPr>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <cols>
+    <col min="1" max="1" width="4.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="6.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="19.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="15.71" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="18.71" hidden="0" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" t="n">
+        <v>147479561921.3</v>
+      </c>
+      <c r="E2" t="n">
+        <v>6.63</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" t="n">
+        <v>65630254046.8</v>
+      </c>
+      <c r="E3" t="n">
+        <v>2.95</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4" t="n">
+        <v>48849976023</v>
+      </c>
+      <c r="E4" t="n">
+        <v>2.19</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" t="n">
+        <v>41747093211.3</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1.88</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" t="s">
+        <v>16</v>
+      </c>
+      <c r="D6" t="n">
+        <v>29910961325.2</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1.34</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D7" t="n">
+        <v>25751382183.8</v>
+      </c>
+      <c r="E7" t="n">
+        <v>1.16</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>28</v>
+      </c>
+      <c r="C8" t="s">
+        <v>29</v>
+      </c>
+      <c r="D8" t="n">
+        <v>24954367666.2</v>
+      </c>
+      <c r="E8" t="n">
+        <v>1.12</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>23</v>
+      </c>
+      <c r="C9" t="s">
+        <v>24</v>
+      </c>
+      <c r="D9" t="n">
+        <v>20730381620.4</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.93</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>25</v>
+      </c>
+      <c r="C10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10" t="n">
+        <v>19080434180</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.86</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>19</v>
+      </c>
+      <c r="C11" t="s">
+        <v>20</v>
+      </c>
+      <c r="D11" t="n">
+        <v>18792907963.2</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.84</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+  <legacyDrawing r:id="rIdvml"/>
+  <tableParts count="1">
+    <tablePart r:id="rId6"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <sheetPr>
     <tabColor rgb="FFBAB0AC"/>
@@ -1572,21 +2367,21 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="B2" t="n">
         <v>16835</v>
@@ -1600,7 +2395,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="B3" t="n">
         <v>13006</v>
@@ -1614,7 +2409,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="B4" t="n">
         <v>10653</v>
@@ -1628,7 +2423,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="B5" t="n">
         <v>9935</v>
@@ -1642,7 +2437,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="B6" t="n">
         <v>6678</v>
@@ -1656,7 +2451,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="B7" t="n">
         <v>6528</v>
@@ -1670,7 +2465,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="B8" t="n">
         <v>6015</v>
@@ -1684,7 +2479,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="B9" t="n">
         <v>5820</v>
@@ -1698,7 +2493,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="B10" t="n">
         <v>5486</v>
@@ -1712,7 +2507,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="B11" t="n">
         <v>5017</v>
@@ -1726,7 +2521,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="B12" t="n">
         <v>4863</v>
@@ -1740,7 +2535,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="B13" t="n">
         <v>4547</v>
@@ -1754,7 +2549,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="B14" t="n">
         <v>4268</v>
@@ -1768,7 +2563,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="B15" t="n">
         <v>4240</v>
@@ -1782,7 +2577,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="B16" t="n">
         <v>4215</v>
@@ -1796,7 +2591,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="B17" t="n">
         <v>3879</v>
@@ -1810,7 +2605,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="B18" t="n">
         <v>3716</v>
@@ -1824,7 +2619,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="B19" t="n">
         <v>3507</v>
@@ -1838,7 +2633,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="B20" t="n">
         <v>2521</v>
@@ -1852,7 +2647,7 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="B21" t="n">
         <v>2519</v>
@@ -1869,25 +2664,661 @@
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
   <legacyDrawing r:id="rIdvml"/>
   <tableParts count="1">
-    <tablePart r:id="rId5"/>
+    <tablePart r:id="rId7"/>
   </tableParts>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <sheetPr>
-    <tabColor rgb="FFFF9DA7"/>
+    <tabColor rgb="FFBAB0AC"/>
+  </sheetPr>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <cols>
+    <col min="1" max="1" width="16.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="15.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="13.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="19.71" hidden="0" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B2" t="n">
+        <v>15885.2</v>
+      </c>
+      <c r="C2" t="n">
+        <v>134</v>
+      </c>
+      <c r="D2" t="n">
+        <v>14.11</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B3" t="n">
+        <v>12318.8</v>
+      </c>
+      <c r="C3" t="n">
+        <v>103</v>
+      </c>
+      <c r="D3" t="n">
+        <v>10.94</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B4" t="n">
+        <v>9866.4</v>
+      </c>
+      <c r="C4" t="n">
+        <v>112</v>
+      </c>
+      <c r="D4" t="n">
+        <v>8.76</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>36</v>
+      </c>
+      <c r="B5" t="n">
+        <v>9056</v>
+      </c>
+      <c r="C5" t="n">
+        <v>97</v>
+      </c>
+      <c r="D5" t="n">
+        <v>8.04</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>38</v>
+      </c>
+      <c r="B6" t="n">
+        <v>6194.5</v>
+      </c>
+      <c r="C6" t="n">
+        <v>106</v>
+      </c>
+      <c r="D6" t="n">
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>37</v>
+      </c>
+      <c r="B7" t="n">
+        <v>6158.6</v>
+      </c>
+      <c r="C7" t="n">
+        <v>90</v>
+      </c>
+      <c r="D7" t="n">
+        <v>5.47</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>40</v>
+      </c>
+      <c r="B8" t="n">
+        <v>5382.4</v>
+      </c>
+      <c r="C8" t="n">
+        <v>72</v>
+      </c>
+      <c r="D8" t="n">
+        <v>4.78</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>39</v>
+      </c>
+      <c r="B9" t="n">
+        <v>5300.9</v>
+      </c>
+      <c r="C9" t="n">
+        <v>106</v>
+      </c>
+      <c r="D9" t="n">
+        <v>4.71</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>41</v>
+      </c>
+      <c r="B10" t="n">
+        <v>4944.1</v>
+      </c>
+      <c r="C10" t="n">
+        <v>68</v>
+      </c>
+      <c r="D10" t="n">
+        <v>4.39</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>42</v>
+      </c>
+      <c r="B11" t="n">
+        <v>4792.8</v>
+      </c>
+      <c r="C11" t="n">
+        <v>100</v>
+      </c>
+      <c r="D11" t="n">
+        <v>4.26</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>43</v>
+      </c>
+      <c r="B12" t="n">
+        <v>4455.7</v>
+      </c>
+      <c r="C12" t="n">
+        <v>74</v>
+      </c>
+      <c r="D12" t="n">
+        <v>3.96</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>46</v>
+      </c>
+      <c r="B13" t="n">
+        <v>4012.6</v>
+      </c>
+      <c r="C13" t="n">
+        <v>78</v>
+      </c>
+      <c r="D13" t="n">
+        <v>3.56</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s">
+        <v>44</v>
+      </c>
+      <c r="B14" t="n">
+        <v>3922.1</v>
+      </c>
+      <c r="C14" t="n">
+        <v>99</v>
+      </c>
+      <c r="D14" t="n">
+        <v>3.48</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s">
+        <v>47</v>
+      </c>
+      <c r="B15" t="n">
+        <v>3729.8</v>
+      </c>
+      <c r="C15" t="n">
+        <v>60</v>
+      </c>
+      <c r="D15" t="n">
+        <v>3.31</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
+        <v>48</v>
+      </c>
+      <c r="B16" t="n">
+        <v>3662.2</v>
+      </c>
+      <c r="C16" t="n">
+        <v>84</v>
+      </c>
+      <c r="D16" t="n">
+        <v>3.25</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>49</v>
+      </c>
+      <c r="B17" t="n">
+        <v>3451.3</v>
+      </c>
+      <c r="C17" t="n">
+        <v>86</v>
+      </c>
+      <c r="D17" t="n">
+        <v>3.07</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s">
+        <v>50</v>
+      </c>
+      <c r="B18" t="n">
+        <v>3299.9</v>
+      </c>
+      <c r="C18" t="n">
+        <v>48</v>
+      </c>
+      <c r="D18" t="n">
+        <v>2.93</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s">
+        <v>52</v>
+      </c>
+      <c r="B19" t="n">
+        <v>2330.4</v>
+      </c>
+      <c r="C19" t="n">
+        <v>56</v>
+      </c>
+      <c r="D19" t="n">
+        <v>2.07</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s">
+        <v>51</v>
+      </c>
+      <c r="B20" t="n">
+        <v>2282.3</v>
+      </c>
+      <c r="C20" t="n">
+        <v>48</v>
+      </c>
+      <c r="D20" t="n">
+        <v>2.03</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s">
+        <v>45</v>
+      </c>
+      <c r="B21" t="n">
+        <v>1526.9</v>
+      </c>
+      <c r="C21" t="n">
+        <v>20</v>
+      </c>
+      <c r="D21" t="n">
+        <v>1.36</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+  <legacyDrawing r:id="rIdvml"/>
+  <tableParts count="1">
+    <tablePart r:id="rId8"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <sheetPr>
+    <tabColor rgb="FFBAB0AC"/>
+  </sheetPr>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <cols>
+    <col min="1" max="1" width="16.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="15.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="13.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="19.71" hidden="0" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B2" t="n">
+        <v>138000000000</v>
+      </c>
+      <c r="C2" t="n">
+        <v>83</v>
+      </c>
+      <c r="D2" t="n">
+        <v>6.2</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>47</v>
+      </c>
+      <c r="B3" t="n">
+        <v>134000000000</v>
+      </c>
+      <c r="C3" t="n">
+        <v>60</v>
+      </c>
+      <c r="D3" t="n">
+        <v>6.02</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B4" t="n">
+        <v>129000000000</v>
+      </c>
+      <c r="C4" t="n">
+        <v>103</v>
+      </c>
+      <c r="D4" t="n">
+        <v>5.8</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>39</v>
+      </c>
+      <c r="B5" t="n">
+        <v>129000000000</v>
+      </c>
+      <c r="C5" t="n">
+        <v>103</v>
+      </c>
+      <c r="D5" t="n">
+        <v>5.8</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>49</v>
+      </c>
+      <c r="B6" t="n">
+        <v>126000000000</v>
+      </c>
+      <c r="C6" t="n">
+        <v>85</v>
+      </c>
+      <c r="D6" t="n">
+        <v>5.66</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>50</v>
+      </c>
+      <c r="B7" t="n">
+        <v>126000000000</v>
+      </c>
+      <c r="C7" t="n">
+        <v>47</v>
+      </c>
+      <c r="D7" t="n">
+        <v>5.66</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>51</v>
+      </c>
+      <c r="B8" t="n">
+        <v>117000000000</v>
+      </c>
+      <c r="C8" t="n">
+        <v>48</v>
+      </c>
+      <c r="D8" t="n">
+        <v>5.26</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>44</v>
+      </c>
+      <c r="B9" t="n">
+        <v>117000000000</v>
+      </c>
+      <c r="C9" t="n">
+        <v>96</v>
+      </c>
+      <c r="D9" t="n">
+        <v>5.26</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>34</v>
+      </c>
+      <c r="B10" t="n">
+        <v>114000000000</v>
+      </c>
+      <c r="C10" t="n">
+        <v>87</v>
+      </c>
+      <c r="D10" t="n">
+        <v>5.12</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>33</v>
+      </c>
+      <c r="B11" t="n">
+        <v>112000000000</v>
+      </c>
+      <c r="C11" t="n">
+        <v>110</v>
+      </c>
+      <c r="D11" t="n">
+        <v>5.03</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>45</v>
+      </c>
+      <c r="B12" t="n">
+        <v>110000000000</v>
+      </c>
+      <c r="C12" t="n">
+        <v>20</v>
+      </c>
+      <c r="D12" t="n">
+        <v>4.94</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>37</v>
+      </c>
+      <c r="B13" t="n">
+        <v>108000000000</v>
+      </c>
+      <c r="C13" t="n">
+        <v>87</v>
+      </c>
+      <c r="D13" t="n">
+        <v>4.85</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s">
+        <v>46</v>
+      </c>
+      <c r="B14" t="n">
+        <v>108000000000</v>
+      </c>
+      <c r="C14" t="n">
+        <v>78</v>
+      </c>
+      <c r="D14" t="n">
+        <v>4.85</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s">
+        <v>40</v>
+      </c>
+      <c r="B15" t="n">
+        <v>105000000000</v>
+      </c>
+      <c r="C15" t="n">
+        <v>61</v>
+      </c>
+      <c r="D15" t="n">
+        <v>4.72</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
+        <v>43</v>
+      </c>
+      <c r="B16" t="n">
+        <v>98000000000</v>
+      </c>
+      <c r="C16" t="n">
+        <v>73</v>
+      </c>
+      <c r="D16" t="n">
+        <v>4.4</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>42</v>
+      </c>
+      <c r="B17" t="n">
+        <v>97000000000</v>
+      </c>
+      <c r="C17" t="n">
+        <v>96</v>
+      </c>
+      <c r="D17" t="n">
+        <v>4.36</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s">
+        <v>36</v>
+      </c>
+      <c r="B18" t="n">
+        <v>94000000000</v>
+      </c>
+      <c r="C18" t="n">
+        <v>85</v>
+      </c>
+      <c r="D18" t="n">
+        <v>4.22</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s">
+        <v>41</v>
+      </c>
+      <c r="B19" t="n">
+        <v>91000000000</v>
+      </c>
+      <c r="C19" t="n">
+        <v>64</v>
+      </c>
+      <c r="D19" t="n">
+        <v>4.09</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s">
+        <v>52</v>
+      </c>
+      <c r="B20" t="n">
+        <v>89000000000</v>
+      </c>
+      <c r="C20" t="n">
+        <v>55</v>
+      </c>
+      <c r="D20" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s">
+        <v>38</v>
+      </c>
+      <c r="B21" t="n">
+        <v>84000000000</v>
+      </c>
+      <c r="C21" t="n">
+        <v>97</v>
+      </c>
+      <c r="D21" t="n">
+        <v>3.77</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+  <legacyDrawing r:id="rIdvml"/>
+  <tableParts count="1">
+    <tablePart r:id="rId9"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <sheetPr>
+    <tabColor rgb="FFAF7AA1"/>
   </sheetPr>
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
     <col min="1" max="1" width="24.71" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="15.71" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="126.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="29.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="162.71" hidden="0" customWidth="1"/>
     <col min="4" max="4" width="32.71" hidden="0" customWidth="1"/>
-    <col min="5" max="5" width="15.71" hidden="0" customWidth="1"/>
-    <col min="6" max="6" width="14.71" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="156.71" hidden="0" customWidth="1"/>
+    <col min="6" max="6" width="32.71" hidden="0" customWidth="1"/>
     <col min="7" max="7" width="130.71" hidden="0" customWidth="1"/>
     <col min="8" max="8" width="32.71" hidden="0" customWidth="1"/>
     <col min="9" max="9" width="95.71" hidden="0" customWidth="1"/>
@@ -1904,86 +3335,86 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="B2" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="C2" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="D2" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="E2"/>
       <c r="F2"/>
       <c r="G2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="H2" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="I2" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="J2" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="K2"/>
       <c r="L2"/>
@@ -2000,10 +3431,114 @@
         <v>10</v>
       </c>
       <c r="Q2" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="R2" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>80</v>
+      </c>
+      <c r="B3" t="s">
+        <v>90</v>
+      </c>
+      <c r="C3" t="s">
+        <v>91</v>
+      </c>
+      <c r="D3" t="s">
+        <v>92</v>
+      </c>
+      <c r="E3" t="s">
+        <v>93</v>
+      </c>
+      <c r="F3" t="s">
+        <v>94</v>
+      </c>
+      <c r="G3" t="s">
         <v>84</v>
+      </c>
+      <c r="H3" t="s">
+        <v>85</v>
+      </c>
+      <c r="I3" t="s">
+        <v>86</v>
+      </c>
+      <c r="J3" t="s">
+        <v>87</v>
+      </c>
+      <c r="K3"/>
+      <c r="L3"/>
+      <c r="M3" t="n">
+        <v>232</v>
+      </c>
+      <c r="N3" t="n">
+        <v>232</v>
+      </c>
+      <c r="O3" t="n">
+        <v>232</v>
+      </c>
+      <c r="P3" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>88</v>
+      </c>
+      <c r="R3" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>80</v>
+      </c>
+      <c r="B4" t="s">
+        <v>95</v>
+      </c>
+      <c r="C4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D4" t="s">
+        <v>97</v>
+      </c>
+      <c r="E4" t="s">
+        <v>98</v>
+      </c>
+      <c r="F4" t="s">
+        <v>99</v>
+      </c>
+      <c r="G4" t="s">
+        <v>84</v>
+      </c>
+      <c r="H4" t="s">
+        <v>85</v>
+      </c>
+      <c r="I4" t="s">
+        <v>86</v>
+      </c>
+      <c r="J4" t="s">
+        <v>87</v>
+      </c>
+      <c r="K4"/>
+      <c r="L4"/>
+      <c r="M4" t="n">
+        <v>232</v>
+      </c>
+      <c r="N4" t="n">
+        <v>232</v>
+      </c>
+      <c r="O4" t="n">
+        <v>232</v>
+      </c>
+      <c r="P4" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>88</v>
+      </c>
+      <c r="R4" t="s">
+        <v>89</v>
       </c>
     </row>
   </sheetData>
@@ -2011,381 +3546,579 @@
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
   <legacyDrawing r:id="rIdvml"/>
   <tableParts count="1">
-    <tablePart r:id="rId6"/>
+    <tablePart r:id="rId10"/>
   </tableParts>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <sheetPr>
-    <tabColor rgb="FF9C755F"/>
+    <tabColor rgb="FFFF9DA7"/>
   </sheetPr>
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col min="1" max="1" width="16.71" hidden="0" customWidth="1"/>
+    <col min="1" max="1" width="25.71" hidden="0" customWidth="1"/>
     <col min="2" max="2" width="21.71" hidden="0" customWidth="1"/>
     <col min="3" max="3" width="250.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>85</v>
+        <v>100</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>86</v>
+        <v>101</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>87</v>
+        <v>102</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>88</v>
+        <v>103</v>
       </c>
       <c r="B2" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="C2" t="s">
-        <v>89</v>
+        <v>104</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>88</v>
+        <v>103</v>
       </c>
       <c r="B3" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C3" t="s">
-        <v>90</v>
+        <v>105</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>88</v>
+        <v>103</v>
       </c>
       <c r="B4" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="C4" t="s">
-        <v>91</v>
+        <v>106</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>88</v>
+        <v>103</v>
       </c>
       <c r="B5" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="C5" t="s">
-        <v>92</v>
+        <v>107</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>88</v>
+        <v>103</v>
       </c>
       <c r="B6" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="C6" t="s">
-        <v>93</v>
+        <v>108</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>88</v>
+        <v>103</v>
       </c>
       <c r="B7" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="C7" t="s">
-        <v>94</v>
+        <v>109</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>88</v>
+        <v>103</v>
       </c>
       <c r="B8" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="C8" t="s">
-        <v>95</v>
+        <v>110</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>88</v>
+        <v>103</v>
       </c>
       <c r="B9" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="C9" t="s">
-        <v>96</v>
+        <v>111</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>88</v>
+        <v>103</v>
       </c>
       <c r="B10" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="C10" t="s">
-        <v>97</v>
+        <v>112</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>88</v>
+        <v>103</v>
       </c>
       <c r="B11" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="C11" t="s">
-        <v>98</v>
+        <v>113</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>88</v>
+        <v>103</v>
       </c>
       <c r="B12" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="C12" t="s">
-        <v>99</v>
+        <v>114</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>88</v>
+        <v>103</v>
       </c>
       <c r="B13" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="C13" t="s">
-        <v>100</v>
+        <v>115</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>88</v>
+        <v>103</v>
       </c>
       <c r="B14" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="C14" t="s">
-        <v>101</v>
+        <v>116</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>88</v>
+        <v>103</v>
       </c>
       <c r="B15" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="C15" t="s">
-        <v>102</v>
+        <v>117</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>88</v>
+        <v>103</v>
       </c>
       <c r="B16" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="C16" t="s">
-        <v>103</v>
+        <v>118</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>88</v>
+        <v>103</v>
       </c>
       <c r="B17" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="C17" t="s">
-        <v>104</v>
+        <v>119</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>88</v>
+        <v>103</v>
       </c>
       <c r="B18" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="C18" t="s">
-        <v>105</v>
+        <v>120</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>88</v>
+        <v>103</v>
       </c>
       <c r="B19" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="C19" t="s">
-        <v>106</v>
+        <v>121</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>107</v>
+        <v>122</v>
       </c>
       <c r="B20" t="s">
         <v>0</v>
       </c>
       <c r="C20" t="s">
-        <v>108</v>
+        <v>123</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>107</v>
+        <v>122</v>
       </c>
       <c r="B21" t="s">
         <v>1</v>
       </c>
       <c r="C21" t="s">
-        <v>109</v>
+        <v>124</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>107</v>
+        <v>122</v>
       </c>
       <c r="B22" t="s">
         <v>2</v>
       </c>
       <c r="C22" t="s">
-        <v>110</v>
+        <v>125</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>107</v>
+        <v>122</v>
       </c>
       <c r="B23" t="s">
         <v>3</v>
       </c>
       <c r="C23" t="s">
-        <v>111</v>
+        <v>126</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>107</v>
+        <v>122</v>
       </c>
       <c r="B24" t="s">
         <v>4</v>
       </c>
       <c r="C24" t="s">
-        <v>112</v>
+        <v>127</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>113</v>
+        <v>128</v>
       </c>
       <c r="B25" t="s">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="C25" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>113</v>
+        <v>128</v>
       </c>
       <c r="B26" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C26" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>113</v>
+        <v>128</v>
       </c>
       <c r="B27" t="s">
-        <v>26</v>
+        <v>2</v>
       </c>
       <c r="C27" t="s">
-        <v>116</v>
+        <v>125</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>113</v>
+        <v>128</v>
       </c>
       <c r="B28" t="s">
-        <v>27</v>
+        <v>3</v>
       </c>
       <c r="C28" t="s">
-        <v>117</v>
+        <v>126</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>118</v>
+        <v>128</v>
       </c>
       <c r="B29" t="s">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C29" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>118</v>
+        <v>129</v>
       </c>
       <c r="B30" t="s">
-        <v>48</v>
+        <v>0</v>
       </c>
       <c r="C30" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>118</v>
+        <v>129</v>
       </c>
       <c r="B31" t="s">
-        <v>49</v>
+        <v>1</v>
       </c>
       <c r="C31" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>118</v>
+        <v>129</v>
       </c>
       <c r="B32" t="s">
-        <v>50</v>
+        <v>2</v>
       </c>
       <c r="C32" t="s">
-        <v>122</v>
+        <v>125</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="s">
+        <v>129</v>
+      </c>
+      <c r="B33" t="s">
+        <v>3</v>
+      </c>
+      <c r="C33" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="s">
+        <v>129</v>
+      </c>
+      <c r="B34" t="s">
+        <v>4</v>
+      </c>
+      <c r="C34" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="s">
+        <v>130</v>
+      </c>
+      <c r="B35" t="s">
+        <v>30</v>
+      </c>
+      <c r="C35" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="s">
+        <v>130</v>
+      </c>
+      <c r="B36" t="s">
+        <v>3</v>
+      </c>
+      <c r="C36" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="s">
+        <v>130</v>
+      </c>
+      <c r="B37" t="s">
+        <v>31</v>
+      </c>
+      <c r="C37" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="s">
+        <v>130</v>
+      </c>
+      <c r="B38" t="s">
+        <v>32</v>
+      </c>
+      <c r="C38" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="s">
+        <v>135</v>
+      </c>
+      <c r="B39" t="s">
+        <v>30</v>
+      </c>
+      <c r="C39" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="s">
+        <v>135</v>
+      </c>
+      <c r="B40" t="s">
+        <v>3</v>
+      </c>
+      <c r="C40" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="s">
+        <v>135</v>
+      </c>
+      <c r="B41" t="s">
+        <v>31</v>
+      </c>
+      <c r="C41" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="s">
+        <v>135</v>
+      </c>
+      <c r="B42" t="s">
+        <v>32</v>
+      </c>
+      <c r="C42" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="s">
+        <v>136</v>
+      </c>
+      <c r="B43" t="s">
+        <v>30</v>
+      </c>
+      <c r="C43" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="s">
+        <v>136</v>
+      </c>
+      <c r="B44" t="s">
+        <v>3</v>
+      </c>
+      <c r="C44" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="s">
+        <v>136</v>
+      </c>
+      <c r="B45" t="s">
+        <v>31</v>
+      </c>
+      <c r="C45" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="s">
+        <v>136</v>
+      </c>
+      <c r="B46" t="s">
+        <v>32</v>
+      </c>
+      <c r="C46" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="s">
+        <v>137</v>
+      </c>
+      <c r="B47" t="s">
+        <v>0</v>
+      </c>
+      <c r="C47" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="s">
+        <v>137</v>
+      </c>
+      <c r="B48" t="s">
+        <v>53</v>
+      </c>
+      <c r="C48" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="s">
+        <v>137</v>
+      </c>
+      <c r="B49" t="s">
+        <v>54</v>
+      </c>
+      <c r="C49" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="s">
+        <v>137</v>
+      </c>
+      <c r="B50" t="s">
+        <v>55</v>
+      </c>
+      <c r="C50" t="s">
+        <v>141</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
   <tableParts count="1">
-    <tablePart r:id="rId7"/>
+    <tablePart r:id="rId11"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Run every workflow step in the bundled example
</commit_message>
<xml_diff>
--- a/example/reference_results/9_phyloseq_object/GTDB/phyloseq_summary_gtdb.xlsx
+++ b/example/reference_results/9_phyloseq_object/GTDB/phyloseq_summary_gtdb.xlsx
@@ -688,7 +688,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="144">
   <si>
     <t xml:space="preserve">Rank</t>
   </si>
@@ -930,7 +930,7 @@
     <t xml:space="preserve">R_Version</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-09-29 15:16:34 CEST</t>
+    <t xml:space="preserve">2026-09-29 15:28:05 CEST</t>
   </si>
   <si>
     <t xml:space="preserve">GTDB_raw_counts</t>
@@ -954,6 +954,12 @@
     <t xml:space="preserve">8a016686bccd6a49787b7859a1de0436</t>
   </si>
   <si>
+    <t xml:space="preserve">/Users/amro/Documents/workflows/DADA2_16S_Illumina_PairedEnd_Workflow/example/run_results/6_phylogenetic_tree/phylogenetic_tree.nwk</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2a0c61f68343e387fae4c899fc2608ae</t>
+  </si>
+  <si>
     <t xml:space="preserve">1.52.0</t>
   </si>
   <si>
@@ -972,7 +978,7 @@
     <t xml:space="preserve">/Users/amro/Documents/workflows/DADA2_16S_Illumina_PairedEnd_Workflow/example/run_results/7_copy_number_correction/copy_number_correction_summary.xlsx</t>
   </si>
   <si>
-    <t xml:space="preserve">143355f48ec0fd4be6486a49b09480fa</t>
+    <t xml:space="preserve">758b23ed2eab74bcc906b02359bb0315</t>
   </si>
   <si>
     <t xml:space="preserve">GTDB_microbial_load_corrected</t>
@@ -987,7 +993,7 @@
     <t xml:space="preserve">/Users/amro/Documents/workflows/DADA2_16S_Illumina_PairedEnd_Workflow/example/run_results/8_microbial_load_correction/microbial_load_correction_summary.xlsx</t>
   </si>
   <si>
-    <t xml:space="preserve">bd25f596934f17d031f57b031d8971ab</t>
+    <t xml:space="preserve">7113c7d14ce8e4f206effb461f420452</t>
   </si>
   <si>
     <t xml:space="preserve">Sheet</t>
@@ -3171,13 +3177,13 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>37</v>
+        <v>46</v>
       </c>
       <c r="B13" t="n">
         <v>108000000000</v>
       </c>
       <c r="C13" t="n">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="D13" t="n">
         <v>4.85</v>
@@ -3185,13 +3191,13 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="B14" t="n">
         <v>108000000000</v>
       </c>
       <c r="C14" t="n">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="D14" t="n">
         <v>4.85</v>
@@ -3323,8 +3329,8 @@
     <col min="8" max="8" width="32.71" hidden="0" customWidth="1"/>
     <col min="9" max="9" width="95.71" hidden="0" customWidth="1"/>
     <col min="10" max="10" width="32.71" hidden="0" customWidth="1"/>
-    <col min="11" max="11" width="9.71" hidden="0" customWidth="1"/>
-    <col min="12" max="12" width="8.71" hidden="0" customWidth="1"/>
+    <col min="11" max="11" width="131.71" hidden="0" customWidth="1"/>
+    <col min="12" max="12" width="32.71" hidden="0" customWidth="1"/>
     <col min="13" max="13" width="10.71" hidden="0" customWidth="1"/>
     <col min="14" max="14" width="21.71" hidden="0" customWidth="1"/>
     <col min="15" max="15" width="10.71" hidden="0" customWidth="1"/>
@@ -3416,8 +3422,12 @@
       <c r="J2" t="s">
         <v>87</v>
       </c>
-      <c r="K2"/>
-      <c r="L2"/>
+      <c r="K2" t="s">
+        <v>88</v>
+      </c>
+      <c r="L2" t="s">
+        <v>89</v>
+      </c>
       <c r="M2" t="n">
         <v>232</v>
       </c>
@@ -3431,10 +3441,10 @@
         <v>10</v>
       </c>
       <c r="Q2" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="R2" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="3">
@@ -3442,19 +3452,19 @@
         <v>80</v>
       </c>
       <c r="B3" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C3" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="D3" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="E3" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="F3" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="G3" t="s">
         <v>84</v>
@@ -3468,8 +3478,12 @@
       <c r="J3" t="s">
         <v>87</v>
       </c>
-      <c r="K3"/>
-      <c r="L3"/>
+      <c r="K3" t="s">
+        <v>88</v>
+      </c>
+      <c r="L3" t="s">
+        <v>89</v>
+      </c>
       <c r="M3" t="n">
         <v>232</v>
       </c>
@@ -3483,10 +3497,10 @@
         <v>10</v>
       </c>
       <c r="Q3" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="R3" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="4">
@@ -3494,19 +3508,19 @@
         <v>80</v>
       </c>
       <c r="B4" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C4" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D4" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E4" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="F4" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="G4" t="s">
         <v>84</v>
@@ -3520,8 +3534,12 @@
       <c r="J4" t="s">
         <v>87</v>
       </c>
-      <c r="K4"/>
-      <c r="L4"/>
+      <c r="K4" t="s">
+        <v>88</v>
+      </c>
+      <c r="L4" t="s">
+        <v>89</v>
+      </c>
       <c r="M4" t="n">
         <v>232</v>
       </c>
@@ -3535,10 +3553,10 @@
         <v>10</v>
       </c>
       <c r="Q4" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="R4" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
   </sheetData>
@@ -3566,552 +3584,552 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B2" t="s">
         <v>62</v>
       </c>
       <c r="C2" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B3" t="s">
         <v>63</v>
       </c>
       <c r="C3" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B4" t="s">
         <v>64</v>
       </c>
       <c r="C4" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B5" t="s">
         <v>65</v>
       </c>
       <c r="C5" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B6" t="s">
         <v>66</v>
       </c>
       <c r="C6" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B7" t="s">
         <v>67</v>
       </c>
       <c r="C7" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B8" t="s">
         <v>68</v>
       </c>
       <c r="C8" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B9" t="s">
         <v>69</v>
       </c>
       <c r="C9" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B10" t="s">
         <v>70</v>
       </c>
       <c r="C10" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B11" t="s">
         <v>71</v>
       </c>
       <c r="C11" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B12" t="s">
         <v>72</v>
       </c>
       <c r="C12" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B13" t="s">
         <v>73</v>
       </c>
       <c r="C13" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B14" t="s">
         <v>74</v>
       </c>
       <c r="C14" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B15" t="s">
         <v>75</v>
       </c>
       <c r="C15" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B16" t="s">
         <v>76</v>
       </c>
       <c r="C16" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B17" t="s">
         <v>77</v>
       </c>
       <c r="C17" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B18" t="s">
         <v>78</v>
       </c>
       <c r="C18" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B19" t="s">
         <v>79</v>
       </c>
       <c r="C19" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B20" t="s">
         <v>0</v>
       </c>
       <c r="C20" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B21" t="s">
         <v>1</v>
       </c>
       <c r="C21" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B22" t="s">
         <v>2</v>
       </c>
       <c r="C22" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B23" t="s">
         <v>3</v>
       </c>
       <c r="C23" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B24" t="s">
         <v>4</v>
       </c>
       <c r="C24" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B25" t="s">
         <v>0</v>
       </c>
       <c r="C25" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B26" t="s">
         <v>1</v>
       </c>
       <c r="C26" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B27" t="s">
         <v>2</v>
       </c>
       <c r="C27" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B28" t="s">
         <v>3</v>
       </c>
       <c r="C28" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B29" t="s">
         <v>4</v>
       </c>
       <c r="C29" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B30" t="s">
         <v>0</v>
       </c>
       <c r="C30" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B31" t="s">
         <v>1</v>
       </c>
       <c r="C31" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B32" t="s">
         <v>2</v>
       </c>
       <c r="C32" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B33" t="s">
         <v>3</v>
       </c>
       <c r="C33" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B34" t="s">
         <v>4</v>
       </c>
       <c r="C34" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B35" t="s">
         <v>30</v>
       </c>
       <c r="C35" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B36" t="s">
         <v>3</v>
       </c>
       <c r="C36" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B37" t="s">
         <v>31</v>
       </c>
       <c r="C37" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B38" t="s">
         <v>32</v>
       </c>
       <c r="C38" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B39" t="s">
         <v>30</v>
       </c>
       <c r="C39" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B40" t="s">
         <v>3</v>
       </c>
       <c r="C40" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B41" t="s">
         <v>31</v>
       </c>
       <c r="C41" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B42" t="s">
         <v>32</v>
       </c>
       <c r="C42" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B43" t="s">
         <v>30</v>
       </c>
       <c r="C43" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B44" t="s">
         <v>3</v>
       </c>
       <c r="C44" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B45" t="s">
         <v>31</v>
       </c>
       <c r="C45" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B46" t="s">
         <v>32</v>
       </c>
       <c r="C46" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B47" t="s">
         <v>0</v>
       </c>
       <c r="C47" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B48" t="s">
         <v>53</v>
       </c>
       <c r="C48" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B49" t="s">
         <v>54</v>
       </c>
       <c r="C49" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B50" t="s">
         <v>55</v>
       </c>
       <c r="C50" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
     </row>
   </sheetData>

</xml_diff>